<commit_message>
fix cpack and tsp4 examples
</commit_message>
<xml_diff>
--- a/models/cta/results.xlsx
+++ b/models/cta/results.xlsx
@@ -416,41 +416,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="C1" t="inlineStr">
         <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>c2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>c4</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>c5</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>c6</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>c7</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>c8</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>c9</t>
         </is>
@@ -467,20 +472,20 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>20</v>
       </c>
-      <c r="D2" t="n">
-        <v>-22</v>
-      </c>
       <c r="E2" t="n">
+        <v>-25</v>
+      </c>
+      <c r="F2" t="n">
         <v>7</v>
       </c>
       <c r="H2" t="n">
-        <v>17</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-22</v>
+        <v>16</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-18</v>
       </c>
     </row>
     <row r="3">
@@ -494,20 +499,17 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>-22</v>
-      </c>
       <c r="E3" t="n">
+        <v>-30</v>
+      </c>
+      <c r="F3" t="n">
         <v>-7</v>
       </c>
-      <c r="F3" t="n">
-        <v>23</v>
-      </c>
       <c r="G3" t="n">
-        <v>14</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-8</v>
+        <v>24</v>
+      </c>
+      <c r="H3" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -521,17 +523,14 @@
           <t>r3</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>-28</v>
-      </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>-24</v>
       </c>
       <c r="H4" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -545,13 +544,16 @@
           <t>r4</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>44</v>
-      </c>
-      <c r="G5" t="n">
-        <v>13</v>
+      <c r="E5" t="n">
+        <v>55</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
       </c>
       <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
         <v>-57</v>
       </c>
     </row>
@@ -566,19 +568,16 @@
           <t>r5</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>-24</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-33</v>
+      <c r="D6" t="n">
+        <v>-20</v>
       </c>
       <c r="H6" t="n">
+        <v>-32</v>
+      </c>
+      <c r="I6" t="n">
         <v>-36</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>88</v>
       </c>
     </row>
@@ -593,11 +592,11 @@
           <t>total</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>-4</v>
-      </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>-13</v>
+      </c>
+      <c r="J7" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -611,17 +610,20 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>-39</v>
       </c>
-      <c r="D8" t="n">
-        <v>5</v>
-      </c>
       <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
         <v>7</v>
       </c>
       <c r="H8" t="n">
-        <v>27</v>
+        <v>-1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -635,16 +637,16 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>-7</v>
       </c>
-      <c r="F9" t="n">
-        <v>-36</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-14</v>
+      <c r="G9" t="n">
+        <v>-35</v>
       </c>
       <c r="I9" t="n">
+        <v>-15</v>
+      </c>
+      <c r="J9" t="n">
         <v>57</v>
       </c>
     </row>
@@ -659,17 +661,17 @@
           <t>r4</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>35</v>
       </c>
-      <c r="D10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H10" t="n">
-        <v>23</v>
+      <c r="E10" t="n">
+        <v>-2</v>
       </c>
       <c r="I10" t="n">
-        <v>-57</v>
+        <v>20</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-53</v>
       </c>
     </row>
     <row r="11">
@@ -683,10 +685,13 @@
           <t>r5</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>36</v>
+      <c r="G11" t="n">
+        <v>35</v>
       </c>
       <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
         <v>-36</v>
       </c>
     </row>
@@ -701,10 +706,10 @@
           <t>total</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>-4</v>
       </c>
-      <c r="D12" t="n">
+      <c r="J12" t="n">
         <v>4</v>
       </c>
     </row>
@@ -720,16 +725,22 @@
         </is>
       </c>
       <c r="C13" t="n">
+        <v>-1.13686837721616e-13</v>
+      </c>
+      <c r="D13" t="n">
         <v>59</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>7</v>
       </c>
-      <c r="F13" t="n">
-        <v>-5</v>
-      </c>
       <c r="G13" t="n">
-        <v>-61</v>
+        <v>-1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-44</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-21</v>
       </c>
     </row>
     <row r="14">
@@ -743,17 +754,17 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>-87</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>59</v>
       </c>
-      <c r="G14" t="n">
-        <v>14</v>
-      </c>
       <c r="H14" t="n">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="I14" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -767,17 +778,17 @@
           <t>r3</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>-30</v>
       </c>
-      <c r="G15" t="n">
-        <v>74</v>
-      </c>
       <c r="H15" t="n">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="I15" t="n">
-        <v>-88</v>
+        <v>51</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-91</v>
       </c>
     </row>
     <row r="16">
@@ -791,13 +802,13 @@
           <t>r4</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>45</v>
-      </c>
-      <c r="G16" t="n">
-        <v>13</v>
+      <c r="E16" t="n">
+        <v>57</v>
       </c>
       <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
         <v>-58</v>
       </c>
     </row>
@@ -813,15 +824,18 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-24</v>
-      </c>
-      <c r="F17" t="n">
-        <v>-24</v>
+        <v>1.13686837721616e-13</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-20</v>
       </c>
       <c r="G17" t="n">
+        <v>-28</v>
+      </c>
+      <c r="H17" t="n">
         <v>-40</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>88</v>
       </c>
     </row>
@@ -836,11 +850,17 @@
           <t>total</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>35</v>
-      </c>
       <c r="D18" t="n">
-        <v>-35</v>
+        <v>39</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-23</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-13</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="19">
@@ -854,20 +874,20 @@
           <t>r1</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>-34</v>
       </c>
-      <c r="F19" t="n">
-        <v>5</v>
-      </c>
       <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
         <v>61</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>-10</v>
       </c>
-      <c r="I19" t="n">
-        <v>-22</v>
+      <c r="J19" t="n">
+        <v>-18</v>
       </c>
     </row>
     <row r="20">
@@ -881,11 +901,11 @@
           <t>r2</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>65</v>
-      </c>
-      <c r="I20" t="n">
-        <v>-65</v>
+      <c r="E20" t="n">
+        <v>57</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-57</v>
       </c>
     </row>
     <row r="21">
@@ -899,16 +919,16 @@
           <t>r3</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>2</v>
-      </c>
       <c r="G21" t="n">
+        <v>6</v>
+      </c>
+      <c r="H21" t="n">
         <v>-68</v>
       </c>
-      <c r="H21" t="n">
-        <v>-25</v>
-      </c>
       <c r="I21" t="n">
+        <v>-29</v>
+      </c>
+      <c r="J21" t="n">
         <v>91</v>
       </c>
     </row>
@@ -923,11 +943,14 @@
           <t>r4</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="D22" t="n">
         <v>-35</v>
       </c>
-      <c r="H22" t="n">
-        <v>35</v>
+      <c r="I22" t="n">
+        <v>39</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-4</v>
       </c>
     </row>
     <row r="23">
@@ -941,10 +964,10 @@
           <t>r5</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>-7</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>7</v>
       </c>
     </row>
@@ -959,14 +982,14 @@
           <t>total</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="D24" t="n">
         <v>-35</v>
       </c>
-      <c r="D24" t="n">
-        <v>31</v>
-      </c>
-      <c r="I24" t="n">
-        <v>4</v>
+      <c r="E24" t="n">
+        <v>23</v>
+      </c>
+      <c r="J24" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1059,7 +1082,7 @@
         <v>6832</v>
       </c>
       <c r="G2" t="n">
-        <v>4729</v>
+        <v>4726</v>
       </c>
       <c r="H2" t="n">
         <v>2063</v>
@@ -1068,13 +1091,13 @@
         <v>8603</v>
       </c>
       <c r="J2" t="n">
-        <v>5196</v>
+        <v>5212</v>
       </c>
       <c r="K2" t="n">
-        <v>5419</v>
+        <v>5402</v>
       </c>
       <c r="L2" t="n">
-        <v>1750</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="3">
@@ -1098,22 +1121,22 @@
         <v>13763</v>
       </c>
       <c r="G3" t="n">
-        <v>1692</v>
+        <v>1684</v>
       </c>
       <c r="H3" t="n">
         <v>3487</v>
       </c>
       <c r="I3" t="n">
-        <v>4601</v>
+        <v>4602</v>
       </c>
       <c r="J3" t="n">
-        <v>2152</v>
+        <v>2151</v>
       </c>
       <c r="K3" t="n">
         <v>8679</v>
       </c>
       <c r="L3" t="n">
-        <v>1121</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="4">
@@ -1143,16 +1166,16 @@
         <v>5793</v>
       </c>
       <c r="I4" t="n">
-        <v>7214</v>
+        <v>7218</v>
       </c>
       <c r="J4" t="n">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="K4" t="n">
-        <v>3871</v>
+        <v>3874</v>
       </c>
       <c r="L4" t="n">
-        <v>1573</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="5">
@@ -1179,7 +1202,7 @@
         <v>1016</v>
       </c>
       <c r="G5" t="n">
-        <v>2871</v>
+        <v>2882</v>
       </c>
       <c r="H5" t="n">
         <v>5585</v>
@@ -1188,10 +1211,10 @@
         <v>4979</v>
       </c>
       <c r="J5" t="n">
-        <v>6129</v>
+        <v>6117</v>
       </c>
       <c r="K5" t="n">
-        <v>5940</v>
+        <v>5941</v>
       </c>
       <c r="L5" t="n">
         <v>11625</v>
@@ -1215,7 +1238,7 @@
         <v>7346</v>
       </c>
       <c r="E6" t="n">
-        <v>2790</v>
+        <v>2794</v>
       </c>
       <c r="G6" t="n">
         <v>2212</v>
@@ -1224,10 +1247,10 @@
         <v>7493</v>
       </c>
       <c r="I6" t="n">
-        <v>5722</v>
+        <v>5717</v>
       </c>
       <c r="J6" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="K6" t="n">
         <v>628</v>
@@ -1254,7 +1277,7 @@
         <v>37025</v>
       </c>
       <c r="E7" t="n">
-        <v>18891</v>
+        <v>18895</v>
       </c>
       <c r="F7" t="n">
         <v>26305</v>
@@ -1272,10 +1295,10 @@
         <v>17103</v>
       </c>
       <c r="K7" t="n">
-        <v>24537</v>
+        <v>24524</v>
       </c>
       <c r="L7" t="n">
-        <v>17755</v>
+        <v>17764</v>
       </c>
     </row>
     <row r="8">
@@ -1302,16 +1325,16 @@
         <v>3356</v>
       </c>
       <c r="G8" t="n">
-        <v>4072</v>
+        <v>4069</v>
       </c>
       <c r="H8" t="n">
         <v>147</v>
       </c>
       <c r="J8" t="n">
-        <v>3932</v>
+        <v>3931</v>
       </c>
       <c r="K8" t="n">
-        <v>1505</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="9">
@@ -1338,10 +1361,10 @@
         <v>3015</v>
       </c>
       <c r="I9" t="n">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="K9" t="n">
-        <v>3206</v>
+        <v>3205</v>
       </c>
       <c r="L9" t="n">
         <v>1099</v>
@@ -1395,16 +1418,16 @@
         <v>10667</v>
       </c>
       <c r="G11" t="n">
-        <v>2444</v>
+        <v>2443</v>
       </c>
       <c r="J11" t="n">
         <v>2313</v>
       </c>
       <c r="K11" t="n">
-        <v>3001</v>
+        <v>2998</v>
       </c>
       <c r="L11" t="n">
-        <v>7491</v>
+        <v>7495</v>
       </c>
     </row>
     <row r="12">
@@ -1428,10 +1451,10 @@
         <v>4667</v>
       </c>
       <c r="I12" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="J12" t="n">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="K12" t="n">
         <v>628</v>
@@ -1461,7 +1484,7 @@
         <v>12657</v>
       </c>
       <c r="G13" t="n">
-        <v>6516</v>
+        <v>6512</v>
       </c>
       <c r="H13" t="n">
         <v>11507</v>
@@ -1476,7 +1499,7 @@
         <v>8340</v>
       </c>
       <c r="L13" t="n">
-        <v>8590</v>
+        <v>8594</v>
       </c>
     </row>
     <row r="14">
@@ -1500,13 +1523,13 @@
         <v>77</v>
       </c>
       <c r="I14" t="n">
-        <v>7467</v>
+        <v>7471</v>
       </c>
       <c r="J14" t="n">
-        <v>654</v>
+        <v>671</v>
       </c>
       <c r="K14" t="n">
-        <v>3832</v>
+        <v>3811</v>
       </c>
     </row>
     <row r="15">
@@ -1539,10 +1562,10 @@
         <v>1133</v>
       </c>
       <c r="J15" t="n">
-        <v>1844</v>
+        <v>1843</v>
       </c>
       <c r="K15" t="n">
-        <v>5044</v>
+        <v>5045</v>
       </c>
     </row>
     <row r="16">
@@ -1569,13 +1592,13 @@
         <v>514</v>
       </c>
       <c r="J16" t="n">
-        <v>705</v>
+        <v>701</v>
       </c>
       <c r="K16" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="L16" t="n">
-        <v>662</v>
+        <v>659</v>
       </c>
     </row>
     <row r="17">
@@ -1599,7 +1622,7 @@
         <v>1016</v>
       </c>
       <c r="G17" t="n">
-        <v>427</v>
+        <v>439</v>
       </c>
       <c r="H17" t="n">
         <v>3175</v>
@@ -1608,7 +1631,7 @@
         <v>3302</v>
       </c>
       <c r="J17" t="n">
-        <v>3816</v>
+        <v>3804</v>
       </c>
       <c r="K17" t="n">
         <v>992</v>
@@ -1632,10 +1655,10 @@
         <v>1648</v>
       </c>
       <c r="E18" t="n">
-        <v>2790</v>
+        <v>2794</v>
       </c>
       <c r="I18" t="n">
-        <v>2078</v>
+        <v>2074</v>
       </c>
       <c r="J18" t="n">
         <v>686</v>
@@ -1662,13 +1685,13 @@
         <v>5875</v>
       </c>
       <c r="E19" t="n">
-        <v>3388</v>
+        <v>3392</v>
       </c>
       <c r="F19" t="n">
         <v>6950</v>
       </c>
       <c r="G19" t="n">
-        <v>1203</v>
+        <v>1215</v>
       </c>
       <c r="H19" t="n">
         <v>3647</v>
@@ -1680,10 +1703,10 @@
         <v>7705</v>
       </c>
       <c r="K19" t="n">
-        <v>9960</v>
+        <v>9947</v>
       </c>
       <c r="L19" t="n">
-        <v>2348</v>
+        <v>2345</v>
       </c>
     </row>
     <row r="20">
@@ -1713,7 +1736,7 @@
         <v>1916</v>
       </c>
       <c r="I20" t="n">
-        <v>1136</v>
+        <v>1132</v>
       </c>
       <c r="J20" t="n">
         <v>610</v>
@@ -1722,7 +1745,7 @@
         <v>82</v>
       </c>
       <c r="L20" t="n">
-        <v>1750</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="21">
@@ -1743,7 +1766,7 @@
         <v>3222</v>
       </c>
       <c r="G21" t="n">
-        <v>993</v>
+        <v>985</v>
       </c>
       <c r="J21" t="n">
         <v>308</v>
@@ -1752,7 +1775,7 @@
         <v>429</v>
       </c>
       <c r="L21" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22">
@@ -1779,13 +1802,13 @@
         <v>2115</v>
       </c>
       <c r="I22" t="n">
-        <v>4198</v>
+        <v>4202</v>
       </c>
       <c r="J22" t="n">
         <v>346</v>
       </c>
       <c r="K22" t="n">
-        <v>3779</v>
+        <v>3775</v>
       </c>
       <c r="L22" t="n">
         <v>911</v>
@@ -1818,10 +1841,10 @@
         <v>1677</v>
       </c>
       <c r="K23" t="n">
-        <v>1947</v>
+        <v>1951</v>
       </c>
       <c r="L23" t="n">
-        <v>4134</v>
+        <v>4130</v>
       </c>
     </row>
     <row r="24">
@@ -1878,7 +1901,7 @@
         <v>6698</v>
       </c>
       <c r="G25" t="n">
-        <v>7477</v>
+        <v>7469</v>
       </c>
       <c r="H25" t="n">
         <v>9267</v>
@@ -1893,7 +1916,7 @@
         <v>6237</v>
       </c>
       <c r="L25" t="n">
-        <v>6817</v>
+        <v>6825</v>
       </c>
     </row>
   </sheetData>
@@ -1907,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1964,7 +1987,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -2000,11 +2023,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>c8</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -2024,7 +2047,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -2044,7 +2067,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -2084,7 +2107,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -2104,7 +2127,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -2115,16 +2138,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>c9</t>
+          <t>c6</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
@@ -2140,11 +2163,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>c6</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>28</v>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -2160,11 +2183,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>c7</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">
@@ -2175,16 +2198,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>c8</t>
+          <t>c4</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15">
@@ -2195,16 +2218,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>c9</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2220,11 +2243,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>c4</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2240,11 +2263,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>c7</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>13</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="18">
@@ -2255,16 +2278,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>r4</t>
+          <t>r5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>c9</t>
+          <t>c2</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
@@ -2280,11 +2303,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>c2</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
@@ -2300,11 +2323,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>c6</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>5</v>
+          <t>c8</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>36</v>
+      </c>
+      <c r="F20" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -2320,11 +2346,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>c7</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>33</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>88</v>
+      </c>
+      <c r="F21" t="n">
+        <v>88</v>
       </c>
     </row>
     <row r="22">
@@ -2335,7 +2364,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>r5</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2344,10 +2373,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>36</v>
-      </c>
-      <c r="F22" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -2358,7 +2384,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>r5</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2367,21 +2393,18 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>88</v>
-      </c>
-      <c r="F23" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>p1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2390,27 +2413,30 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>39</v>
+      </c>
+      <c r="F24" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>p1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>c9</t>
+          <t>c4</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -2426,14 +2452,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>39</v>
+          <t>c5</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
       </c>
       <c r="F26" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -2449,11 +2475,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>c4</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>5</v>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2469,14 +2495,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29">
@@ -2487,16 +2510,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>c8</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>27</v>
+          <t>c5</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="30">
@@ -2512,11 +2535,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c6</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31">
@@ -2532,11 +2555,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>c6</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32">
@@ -2552,11 +2575,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>c8</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>14</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>57</v>
+      </c>
+      <c r="F32" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="33">
@@ -2567,19 +2593,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>c9</t>
+          <t>c2</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>57</v>
-      </c>
-      <c r="F33" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34">
@@ -2595,11 +2618,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>35</v>
+          <t>c4</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -2615,11 +2638,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>c4</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>1</v>
+          <t>c8</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="36">
@@ -2635,11 +2658,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>c8</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>23</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="37">
@@ -2650,16 +2673,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>r4</t>
+          <t>r5</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>c9</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>57</v>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="38">
@@ -2675,11 +2698,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>c6</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2738,7 +2761,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>c4</t>
+          <t>c9</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -2758,14 +2781,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>c2</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>59</v>
-      </c>
-      <c r="F42" t="n">
-        <v>59</v>
+        <v>-1.13686837721616e-13</v>
       </c>
     </row>
     <row r="43">
@@ -2781,14 +2801,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>c4</t>
+          <t>c2</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="F43" t="n">
-        <v>7</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44">
@@ -2804,11 +2824,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>c6</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>5</v>
+          <t>c4</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>7</v>
+      </c>
+      <c r="F44" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="45">
@@ -2824,11 +2847,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>c7</t>
+          <t>c6</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>61</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -2839,19 +2862,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>c4</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>87</v>
-      </c>
-      <c r="F46" t="n">
-        <v>87</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47">
@@ -2862,19 +2882,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>c6</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>59</v>
-      </c>
-      <c r="F47" t="n">
-        <v>59</v>
+          <t>c8</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="48">
@@ -2890,11 +2907,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>c7</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>14</v>
+          <t>c4</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>87</v>
+      </c>
+      <c r="F48" t="n">
+        <v>87</v>
       </c>
     </row>
     <row r="49">
@@ -2910,11 +2930,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>c8</t>
+          <t>c6</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>14</v>
+        <v>59</v>
+      </c>
+      <c r="F49" t="n">
+        <v>59</v>
       </c>
     </row>
     <row r="50">
@@ -2925,19 +2948,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>c6</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>30</v>
-      </c>
-      <c r="F50" t="n">
-        <v>30</v>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="51">
@@ -2948,19 +2968,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>c7</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>74</v>
-      </c>
-      <c r="F51" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52">
@@ -2976,11 +2993,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>c8</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>44</v>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>30</v>
+      </c>
+      <c r="F52" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="53">
@@ -2996,11 +3016,14 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>c9</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>88</v>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>70</v>
+      </c>
+      <c r="F53" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="54">
@@ -3011,19 +3034,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>r4</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>c4</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>45</v>
-      </c>
-      <c r="F54" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
     </row>
     <row r="55">
@@ -3034,16 +3054,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>r4</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>c7</t>
-        </is>
-      </c>
-      <c r="E55" t="n">
-        <v>13</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="56">
@@ -3059,14 +3079,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>c8</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>58</v>
+          <t>c4</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>57</v>
       </c>
       <c r="F56" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
     </row>
     <row r="57">
@@ -3077,16 +3097,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>r5</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>24</v>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -3097,16 +3117,19 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>r5</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>c6</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>24</v>
+        <v>58</v>
+      </c>
+      <c r="F58" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="59">
@@ -3122,14 +3145,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>c7</t>
+          <t>total</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>40</v>
-      </c>
-      <c r="F59" t="n">
-        <v>40</v>
+        <v>-1.13686837721616e-13</v>
       </c>
     </row>
     <row r="60">
@@ -3145,14 +3165,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>c9</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>88</v>
-      </c>
-      <c r="F60" t="n">
-        <v>88</v>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="61">
@@ -3163,16 +3180,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r5</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>35</v>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="62">
@@ -3183,96 +3200,96 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r5</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>c4</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F62" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p2</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>r5</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>c4</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>34</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>88</v>
       </c>
       <c r="F63" t="n">
-        <v>34</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p2</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>c6</t>
+          <t>c2</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>5</v>
+        <v>39</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p2</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>c7</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>61</v>
+          <t>c4</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>23</v>
       </c>
       <c r="F65" t="n">
-        <v>61</v>
+        <v>17</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3281,21 +3298,18 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>10</v>
-      </c>
-      <c r="F66" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p2</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>total</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3304,7 +3318,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68">
@@ -3315,7 +3329,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3323,11 +3337,11 @@
           <t>c4</t>
         </is>
       </c>
-      <c r="E68" t="n">
-        <v>65</v>
+      <c r="D68" t="n">
+        <v>34</v>
       </c>
       <c r="F68" t="n">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="69">
@@ -3338,16 +3352,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>c9</t>
-        </is>
-      </c>
-      <c r="D69" t="n">
-        <v>65</v>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -3358,16 +3372,19 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>c6</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>61</v>
+      </c>
+      <c r="F70" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="71">
@@ -3378,16 +3395,19 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>c7</t>
+          <t>c8</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>68</v>
+        <v>10</v>
+      </c>
+      <c r="F71" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="72">
@@ -3398,16 +3418,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>c8</t>
+          <t>c9</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73">
@@ -3418,19 +3438,19 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>r3</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>c9</t>
+          <t>c4</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="F73" t="n">
-        <v>91</v>
+        <v>51</v>
       </c>
     </row>
     <row r="74">
@@ -3441,19 +3461,19 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>r4</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>c2</t>
+          <t>c9</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>35</v>
-      </c>
-      <c r="F74" t="n">
-        <v>35</v>
+        <v>57.00000000000011</v>
+      </c>
+      <c r="E74" t="n">
+        <v>1.13686837721616e-13</v>
       </c>
     </row>
     <row r="75">
@@ -3464,16 +3484,16 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>r4</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>c8</t>
+          <t>c6</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
@@ -3484,16 +3504,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>r5</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>c6</t>
+          <t>c7</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>7</v>
+        <v>68</v>
       </c>
     </row>
     <row r="77">
@@ -3504,19 +3524,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>r5</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>c7</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>7</v>
-      </c>
-      <c r="F77" t="n">
-        <v>7</v>
+          <t>c8</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="78">
@@ -3527,16 +3544,19 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r3</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>c2</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>35</v>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>91</v>
+      </c>
+      <c r="F78" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="79">
@@ -3547,16 +3567,19 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>c4</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>31</v>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>35</v>
+      </c>
+      <c r="F79" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="80">
@@ -3567,16 +3590,145 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>r4</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
+          <t>c8</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>r4</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
           <t>c9</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="D81" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>r5</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>c6</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>r5</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>c7</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F83" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>c2</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>c4</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>1.13686837721616e-13</v>
+      </c>
+      <c r="E85" t="n">
+        <v>23.00000000000011</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>total</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>c9</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>-1.13686837721616e-13</v>
+      </c>
+      <c r="E86" t="n">
+        <v>11.99999999999989</v>
       </c>
     </row>
   </sheetData>
@@ -4101,19 +4253,19 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>108.9997356757522</v>
+        <v>130.9997169300914</v>
       </c>
       <c r="E17" t="n">
-        <v>112.0002474635839</v>
+        <v>192.9996069520712</v>
       </c>
       <c r="F17" t="n">
-        <v>134.9997706711292</v>
+        <v>131.9998875260353</v>
       </c>
       <c r="G17" t="n">
-        <v>118.0000137537718</v>
+        <v>145.9997612982988</v>
       </c>
       <c r="H17" t="n">
-        <v>124.0004086866975</v>
+        <v>126.9996631890535</v>
       </c>
     </row>
     <row r="18">
@@ -4133,19 +4285,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E18" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F18" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="G18" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="H18" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>